<commit_message>
Module 1 bank: Section 4 PivotTable questions graded on a static worksheet
Questions now keep every requested view visible (second PivotTable rather
than a changed filter) and ask students to highlight the supporting cells.
Pivot answer workbooks rebuilt with an Answer tab; embeds open on it.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013LuETZtTdHfo8QGmA6xd9C
</commit_message>
<xml_diff>
--- a/practice/answers/q084.xlsx
+++ b/practice/answers/q084.xlsx
@@ -7,13 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="1" r:id="rId3"/>
+    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="1" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,11 +47,22 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="004A7C59"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0024302A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0024302A"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,8 +74,18 @@
         <fgColor rgb="004A7C59"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -71,11 +93,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00A9C4AE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A9C4AE"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A9C4AE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A9C4AE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A9C4AE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A9C4AE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -90,7 +134,24 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -22144,6 +22205,106 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="004A7C59"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Question 39 — Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n"/>
+      <c r="D3" s="11" t="n"/>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>(a)</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Year on Rows, with Yield shown as Average and Count for 2020-2025.</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>(b)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>The lowest average is 2021 (about 49.6 bu/ac); the highest is 2025 (about 68.0). Averages rise after 2021.</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>(c)</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>The variety mix changes by year. Count shows how many reported yields support each annual average.</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>The live PivotTable (and chart, where requested) is on the PivotTable worksheet. The highlighted rows there show the values used in the written answers. The Data worksheet contains the source records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="A9:D10"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -96539,13 +96700,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -96553,127 +96714,120 @@
     <col width="23" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Q84 — Year (2020, 2021, 2022, 2023, 2024, 2025)</t>
-        </is>
-      </c>
-    </row>
+    <row r="1"/>
     <row r="2"/>
-    <row r="3"/>
+    <row r="3">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Values</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Values</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Average of Yield_bu_ac</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Count of Yield_bu_ac</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Average of Yield_bu_ac</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Count of Yield_bu_ac</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>62.40606060606061</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>363</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>62.40606060606061</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>363</v>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>49.64015151515152</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>396</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>49.64015151515152</v>
+        <v>59.76946778711485</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>396</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>59.76946778711485</v>
+        <v>61.41678486997636</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>357</v>
+        <v>423</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>61.41678486997636</v>
+        <v>64.67790973871735</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>64.67790973871735</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>421</v>
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>68.02557077625571</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>438</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>68.02557077625571</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B11" s="8" t="n">
         <v>61.15617180984153</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C11" s="9" t="n">
         <v>2398</v>
       </c>
     </row>

</xml_diff>